<commit_message>
update audit log week 3 slot 5
</commit_message>
<xml_diff>
--- a/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
+++ b/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CN7\SWD392\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CN7\SWD392\ai-audit-log-huanthanh01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7052D5-404E-49E7-8E10-351F0BC928B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAD69BBF-DF04-43B9-826D-7EA89D9413C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week 1&amp;2" sheetId="2" r:id="rId2"/>
-    <sheet name="Assignment 2" sheetId="3" r:id="rId3"/>
+    <sheet name="Week 3" sheetId="3" r:id="rId3"/>
     <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -334,18 +334,220 @@
       <t xml:space="preserve"> Tôi sẽ nghiên cứu thêm cho feature "Kiểm tra nội dung độc hại" thành một Use Case ẩn được &lt;&lt;include&gt;&gt; vào luồng đăng bài. Điều này giúp mô tả rõ ràng nghiệp vụ bảo vệ không gian an toàn cho cộng đồng Gen Z.</t>
     </r>
   </si>
+  <si>
+    <t>Slot 5: Hiểu về chương Static modeling</t>
+  </si>
+  <si>
+    <t>"Giải thích các khái niệm cốt lõi của Static Modeling theo phương pháp COMET trong sách của Hassan Gomaa, bao gồm Class, Attribute và các loại Relationship."</t>
+  </si>
+  <si>
+    <t>"Phân biệt sự khác nhau giữa hai mối quan hệ Whole/Part là Composition và Aggregation trong biểu đồ lớp UML. Cho ví dụ thực tế về hệ thống ATM ngân hàng."</t>
+  </si>
+  <si>
+    <t>"Dựa trên chương 7 sách Software Modeling and Design của Hassan Gomaa, hướng dẫn tôi các bước thiết lập một biểu đồ bối cảnh hệ thống phần mềm (Software System Context Diagram) cho ứng dụng mua sắm trực tuyến."</t>
+  </si>
+  <si>
+    <t>"Entity Class là gì trong Static Modeling? Làm sao để xác định và thiết lập các thuộc tính (Attributes) cho lớp thực thể khi phân tích miền bài toán (Problem Domain)?"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Mô hình hóa tĩnh tập trung vào cấu trúc không đổi của hệ thống. Bao gồm: Lớp (Class) là khuôn mẫu; Thuộc tính (Attribute) là dữ liệu của lớp; và các Mối quan hệ như Association (Liên kết), Whole/Part (Toàn thể/Bộ phận), Generalization (Kế thừa).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nhận ra cấu trúc tĩnh ít thay đổi hơn chức năng hệ thống. Quyết định tập trung xác định thực thể (Entity) trước khi thiết lập phương thức (Operation).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Composition là mối quan hệ mạnh, các phần độc lập (như Card Reader, Cash Dispenser) sinh ra và mất đi cùng với thực thể toàn thể (ATM). Aggregation yếu hơn, các phần có thể tháo rời hoặc thuộc về nhiều tập hợp khác nhau.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Đã hiểu rõ bản chất "ràng buộc vòng đời" của Composition. Cần lưu ý áp dụng đúng ký hiệu hình thoi đặc (Composition) và hình thoi rỗng (Aggregation) khi vẽ sơ đồ lớp.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Bước 1: Xác định biên hệ thống phần mềm. Bước 2: Xác định các lớp bên ngoài (External Classes) như Người dùng, Thiết bị, Hệ thống ngoại vi. Bước 3: Định rõ mối quan hệ và tính đa trị (Multiplicity) giữa chúng với hệ thống.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Thấy được tầm quan trọng của việc phân tách rõ ràng biên giới giữa phần cứng/phần mềm và môi trường ngoài. Sẽ áp dụng các stereotype chuẩn như «external user» hay «external system» để làm rõ sơ đồ.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Lớp thực thể («entity») là lớp lưu trữ thông tin, thường có tính bền vững (persistent). Để xác định thuộc tính, cần tìm các giá trị dữ liệu đặc trưng giúp phân biệt các đối tượng trong lớp (ví dụ: customerId, customerName); nếu một lớp chỉ có một thuộc tính duy nhất thì nên xem xét biến nó thành thuộc tính của lớp khác.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Nhận ra việc thiết lập thuộc tính cho lớp thực thể rất giống với việc thiết kế sơ đồ cơ sở dữ liệu quan hệ. Quyết định sẽ gom các quy tắc nghiệp vụ phức tạp ra một lớp riêng (Business Logic Class) thay vì nhồi nhét hết vào các thuộc tính của Entity Class.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -408,7 +610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -422,7 +624,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -437,19 +639,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -885,7 +1096,7 @@
     <col min="4" max="4" width="51.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
@@ -982,9 +1193,94 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="13.109375" customWidth="1"/>
+    <col min="2" max="2" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="123" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="113.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="148.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="159" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="15"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
update audit log slot 6
</commit_message>
<xml_diff>
--- a/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
+++ b/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CN7\SWD392\ai-audit-log-huanthanh01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAD69BBF-DF04-43B9-826D-7EA89D9413C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47CAF5D-360A-40E7-B05C-3469B4976970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -529,18 +529,172 @@
       <t>: Nhận ra việc thiết lập thuộc tính cho lớp thực thể rất giống với việc thiết kế sơ đồ cơ sở dữ liệu quan hệ. Quyết định sẽ gom các quy tắc nghiệp vụ phức tạp ra một lớp riêng (Business Logic Class) thay vì nhồi nhét hết vào các thuộc tính của Entity Class.</t>
     </r>
   </si>
+  <si>
+    <t>Slot 6: Dynamic Interaction Modeling - Sequence Diagrams (Main Sequence)</t>
+  </si>
+  <si>
+    <t>"Làm thế nào để biểu diễn kịch bản chính (Main Sequence) thành công của một Use Case bằng biểu đồ tuần tự theo chuẩn UML 2? Giải thích cách các đối tượng trao đổi thông điệp từ trên xuống dưới theo thời gian."</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Biểu đồ tuần tự sắp xếp các đối tượng theo chiều ngang với các đường lifeline thẳng đứng đại diện cho trục thời gian. Thông điệp được truyền đi từ trên xuống dưới để thể hiện rõ trình tự thực hiện tuyến tính của kịch bản.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nhận thấy sơ đồ này rất trực quan để giải thích luồng xử lý chuẩn cho các bên liên quan. Quyết định sẽ chọn Use Case cốt lõi của hệ thống để thực hành dựng khung trục thời gian trước.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Theo chuẩn UML 2 được đề cập trong sách của Hassan Gomaa, làm thế nào để biểu diễn các kịch bản rẽ nhánh, điều kiện (alt, opt) và vòng lặp (loop) trên cùng một biểu đồ tuần tự?"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> UML 2 sử dụng các khung tương tác tích hợp (Combined Fragments) với các toán tử như alt (cho điều kiện rẽ nhánh trái ngược), opt (cho tùy chọn có hoặc không) và loop (cho vòng lặp) kèm điều kiện ràng buộc trong dấu ngoặc vuông [ ].
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết Định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Hiểu rằng việc gộp chung các kịch bản lỗi/rẽ nhánh giúp sơ đồ bao quát toàn bộ Use Case nhưng dễ gây rối mắt. Quyết định chỉ dùng các mảnh hợp nhất alt/opt cho những logic thực sự quan trọng.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Làm thế nào để áp dụng các tiêu chí cấu trúc đối tượng (Object Structuring Criteria) nhằm chọn ra đúng các thực thể tham gia và gán thông điệp chính xác trên biểu đồ tuần tự?"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Cần bóc tách từ đặc tả Use Case: lấy Actor kích hoạt làm điểm bắt đầu, ánh xạ các lớp biên (Boundary), điều khiển (Control), và thực thể (Entity) từ mô hình tĩnh vào sơ đồ tuần tự để phân định rõ trách nhiệm truyền tin.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết Định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Nhận thấy mô hình tương tác động chính là cầu nối kiểm tra xem sơ đồ lớp tĩnh trước đó đã thiết kế đủ thuộc tính và quan hệ chưa. Quyết định sẽ luôn đối chiếu hai sơ đồ này song song để đảm bảo tính nhất quán.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -610,7 +764,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -624,7 +778,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -639,31 +793,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1193,16 +1359,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
-    <col min="2" max="2" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.33203125" customWidth="1"/>
     <col min="4" max="4" width="53.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
@@ -1268,17 +1434,57 @@
       <c r="C5" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="15"/>
+      <c r="B6" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="146.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="20"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
commit week4 slot 6
</commit_message>
<xml_diff>
--- a/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
+++ b/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CN7\SWD392\ai-audit-log-huanthanh01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47CAF5D-360A-40E7-B05C-3469B4976970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A231F170-6960-4034-90BA-F643E4F986AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week 1&amp;2" sheetId="2" r:id="rId2"/>
     <sheet name="Week 3" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week 4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="55">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -676,18 +676,226 @@
       <t>: Nhận thấy mô hình tương tác động chính là cầu nối kiểm tra xem sơ đồ lớp tĩnh trước đó đã thiết kế đủ thuộc tính và quan hệ chưa. Quyết định sẽ luôn đối chiếu hai sơ đồ này song song để đảm bảo tính nhất quán.</t>
     </r>
   </si>
+  <si>
+    <t>Slot 6: Hiểu về chương Dynamic modeling</t>
+  </si>
+  <si>
+    <t>"Hãy tóm tắt khái niệm Dynamic Modeling trong kiến trúc phần mềm. Sự khác biệt giữa Dynamic Interaction Modeling và Dynamic State Machine Modeling là gì?"</t>
+  </si>
+  <si>
+    <t>"So sánh Communication Diagram (Sơ đồ giao tiếp) và Sequence Diagram (Sơ đồ tuần tự). Điểm mạnh, điểm yếu và mục đích sử dụng của từng loại là gì?"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Định nghĩa rõ Dynamic Modeling là mô hình hóa hành vi động của hệ thống theo thời gian. Đồng thời, phân biệt rõ hai loại: Dynamic Interaction Modeling tập trung vào sự tương tác/trao đổi thông điệp giữa các object (như Sequence/Communication Diagram), còn Dynamic State Machine Modeling tập trung vào sự thay đổi trạng thái nội tại của một object đơn lẻ (Statechart Diagram).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Nắm vững lý thuyết nền tảng này để áp dụng chính xác vào việc thiết kế sơ đồ thực tế cho hệ thống của dự án; tiếp tục đặt câu hỏi cho AI để lấy ví dụ minh họa bằng code/sơ đồ cụ thể.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Đưa ra bảng so sánh chi tiết giữa hai loại sơ đồ tương tác. Sequence Diagram mạnh về biểu diễn luồng thông điệp theo trình tự thời gian (nhìn rõ thứ tự trước sau). Trong khi đó, Communication Diagram lại mạnh về việc làm nổi bật mối quan hệ cấu trúc tổ chức giữa các đối tượng (nhìn rõ các liên kết mạng lưới). Cả hai đều bổ trợ cho nhau tùy thuộc vào góc nhìn kiến trúc cần ưu tiên.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Hiểu rõ khi nào nên dùng loại sơ đồ nào. Quyết định sẽ ưu tiên dùng Sequence Diagram cho các logic nghiệp vụ phức tạp cần rõ ràng về mặt thời gian, và dùng Communication Diagram khi cần giải thích nhanh mối quan hệ kết nối giữa các subsystem/component cho team.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Phân biệt Stateless Dynamic Interaction Modeling (Mô hình tương tác phi trạng thái) và State-Dependent Dynamic Interaction Modeling (Mô hình tương tác phụ thuộc trạng thái). Nêu các bước thực hiện của từng phương pháp."</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Phân biệt rõ hai phương pháp tiếp cận: Stateless áp dụng cho hệ thống/luồng xử lý không phụ thuộc vào trạng thái trước đó (luồng đi thẳng từ đầu đến cuối dựa trên tham số đầu vào), trong khi State-Dependent áp dụng khi tương tác của hệ thống thay đổi tùy thuộc vào trạng thái hiện tại (cần kết hợp với Statechart Diagram). AI cũng liệt kê tuần tự các bước xây dựng (như xác định tác nhân, kịch bản, xác định trạng thái nền) cho từng loại.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Nắm vững quy trình từng bước của hai phương pháp. Đối với dự án hiện tại, người học quyết định phân loại rõ tính năng nào là Stateless (ví dụ: truy vấn dữ liệu) và tính năng nào là State-Dependent (ví dụ: giỏ hàng, thanh toán) trước khi tiến hành vẽ sơ đồ tương tác nhằm đảm bảo tính chính xác của kiến trúc.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Mô hình tương tác động (Dynamic Interaction Model) thực hiện việc hiện thực hóa Use Case (Use Case Realization) như thế nào? Kịch bản (Scenario) đóng vai trò gì trong việc vẽ sơ đồ?"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot 7: Dynamic Interaction Modeling - Sequence Diagrams </t>
+  </si>
+  <si>
+    <t>Slot 7: Dynamic Interaction Modeling - Sequence Diagrams</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Làm rõ cơ chế hiện thực hóa Use Case (Use Case Realization) bằng cách chuyển đổi các bước mô tả tĩnh trong Use Case thành luồng giao tiếp động giữa các đối tượng (qua Sequence/Communication Diagram). Đồng thời, AI nhấn mạnh Kịch bản (Scenario) đóng vai trò là "bản đặc tả luồng đi cụ thể" (chính hoặc phụ), giúp người thiết kế xác định chính xác các message và thứ tự gọi hàm khi vẽ sơ đồ.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Nắm vững mối quan hệ giữa Use Case, Scenario và Sơ đồ tương tác. Người học quyết định sẽ viết chi tiết kịch bản (gồm luồng chính Main flow và luồng rẽ nhánh Alternative flow) cho các tính năng trọng tâm của dự án trước, tạo tiền đề để vẽ các sơ đồ tương tác chính xác và không bị sót case.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -764,7 +972,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -778,7 +986,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -793,43 +1001,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1481,10 +1692,10 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="20"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="22"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1493,9 +1704,116 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="31.88671875" customWidth="1"/>
+    <col min="3" max="3" width="36.88671875" customWidth="1"/>
+    <col min="4" max="4" width="38.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="243" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="253.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="306" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="302.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="166.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="19"/>
+    </row>
+    <row r="7" spans="1:4" ht="190.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="19"/>
+    </row>
+    <row r="8" spans="1:4" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="19"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
commit week4 slot 7
</commit_message>
<xml_diff>
--- a/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
+++ b/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CN7\SWD392\ai-audit-log-huanthanh01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A231F170-6960-4034-90BA-F643E4F986AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7F2E2EC-2027-4340-90A4-9C1E6FB8C1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="61">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -877,18 +877,169 @@
       <t>: Nắm vững mối quan hệ giữa Use Case, Scenario và Sơ đồ tương tác. Người học quyết định sẽ viết chi tiết kịch bản (gồm luồng chính Main flow và luồng rẽ nhánh Alternative flow) cho các tính năng trọng tâm của dự án trước, tạo tiền đề để vẽ các sơ đồ tương tác chính xác và không bị sót case.</t>
     </r>
   </si>
+  <si>
+    <t>"So sánh Sequence Diagram và Communication Diagram. Sơ đồ nào hiển thị rõ trình tự thời gian hơn, sơ đồ nào hiển thị rõ cấu trúc liên kết hơn? Phương pháp COMET ưu tiên dùng loại nào để thiết kế kiến trúc phần mềm?"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Sequence Diagram hiển thị rõ trình tự thời gian nhờ trục dọc, còn Communication Diagram hiển thị rõ cấu trúc liên kết mạng lưới giữa các đối tượng. Trong phương pháp COMET, Sequence Diagram được ưu tiên sử dụng cho các tương tác phụ thuộc trạng thái (State-Dependent) nhờ khả năng kiểm soát luồng chuyển đổi chặt chẽ, trong khi loại còn lại dùng cho luồng phi trạng thái (Stateless).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Nắm chắc tiêu chí phân biệt và tư duy chọn sơ đồ theo chuẩn COMET. Người học quyết định sẽ ưu tiên sử dụng Sequence Diagram làm công cụ chính để thiết kế kiến trúc phần mềm cho các luồng nghiệp vụ phức tạp của dự án nhằm đảm bảo tính minh bạch về mặt thời gian.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Thế nào là dạng Instance và dạng Generic của Sequence Diagram? Tại sao sách khuyến nghị nên dùng dạng Instance thay vì vẽ một sơ đồ Generic khổng lồ gộp cả vòng lặp và điều kiện rẽ nhánh?"</t>
+  </si>
+  <si>
+    <t>"Dựa vào sách Software Modeling and Design, hãy tạo cho tôi một bảng Reflection Form về chủ đề 'Sequence Diagram' gồm 3 cột: Nội dung Prompt, Phản hồi của AI (tập trung vào cấu trúc, sự khác biệt với Communication Diagram, và các khối alt/loop), và Quyết định của người học."</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Phân biệt rõ Instance form mô tả duy nhất một kịch bản cụ thể (luồng đi thẳng, không rẽ nhánh), giúp sơ đồ cực kỳ dễ đọc. Trong khi đó, Generic form mô tả tất cả các kịch bản có thể xảy ra của một Use Case bằng cách gộp cả các khối điều kiện (alt, opt, loop). Sách khuyến nghị dùng dạng Instance vì một sơ đồ Generic quá lớn sẽ trở nên cực kỳ phức tạp, rối mắt, khó bảo trì và làm mất đi thế mạnh trực quan vốn có của Sequence Diagram.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Thấu hiểu tư duy thiết kế thực tế. Người học quyết định sẽ chia nhỏ các Use Case phức tạp thành nhiều sơ đồ dạng Instance tương ứng với các kịch bản (Scenario) chính/phụ khác nhau, thay vì cố gắng nhồi nhét mọi logic rẽ nhánh vào một sơ đồ duy nhất.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Hệ thống hóa toàn bộ kiến thức cốt lõi về Sequence Diagram từ cuốn sách của Hassan Gomaa thành một bảng Reflection chỉn chu. Nội dung bao gồm việc làm rõ cấu trúc trục thời gian dọc, so sánh thế mạnh với Communication Diagram, và cách dùng các khung tương tác (Interaction Frames) như alt (rẽ nhánh), loop (vòng lặp) để kiểm soát luồng động.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Sử dụng chính bảng tổng hợp này làm biểu mẫu chuẩn (Template) để tự đánh giá và hoàn thiện các nội dung báo cáo học tập/OJT tiếp theo một cách đồng bộ và chuyên nghiệp.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -972,7 +1123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -986,7 +1137,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1001,44 +1152,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1783,35 +1937,47 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="166.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="256.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="19"/>
-    </row>
-    <row r="7" spans="1:4" ht="190.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="310.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="19"/>
-    </row>
-    <row r="8" spans="1:4" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="246" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="19"/>
+      <c r="C8" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>60</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
audit log for week 5
</commit_message>
<xml_diff>
--- a/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
+++ b/AI Audit Log_SE19B06_ThanhAnhHuan_DE190990.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CN7\SWD392\ai-audit-log-huanthanh01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7F2E2EC-2027-4340-90A4-9C1E6FB8C1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86168C86-CA4A-4A4B-AB44-F27F02BF4EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week 1&amp;2" sheetId="2" r:id="rId2"/>
     <sheet name="Week 3" sheetId="3" r:id="rId3"/>
     <sheet name="Week 4" sheetId="4" r:id="rId4"/>
+    <sheet name="Week 5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="77">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -1019,6 +1020,348 @@
         <scheme val="minor"/>
       </rPr>
       <t>: Sử dụng chính bảng tổng hợp này làm biểu mẫu chuẩn (Template) để tự đánh giá và hoàn thiện các nội dung báo cáo học tập/OJT tiếp theo một cách đồng bộ và chuyên nghiệp.</t>
+    </r>
+  </si>
+  <si>
+    <t>Slot 9: Hiểu về chương Dynamic modeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot 10: Dynamic Interaction Modeling - Sequence Diagrams </t>
+  </si>
+  <si>
+    <t>"Trong phương pháp COMET, các thông điệp (messages) trên Sequence Diagram có sự thay đổi như thế nào khi chuyển từ mô hình Phân tích (Analysis model) sang mô hình Thiết kế (Design model)?"</t>
+  </si>
+  <si>
+    <t>"Làm thế nào để biểu diễn cả kịch bản chính (main sequence) và kịch bản thay thế (alternative sequences) trên cùng một Generic Sequence Diagram? Hãy giải thích vai trò của các khối 'alt' và 'loop'."</t>
+  </si>
+  <si>
+    <t>"Trong mô hình tương tác động phụ thuộc trạng thái (State-Dependent Dynamic Interaction Modeling), mối quan hệ giữa một thông điệp (message) trên Sequence Diagram và sự kiện (event)/hành động (action) trên Statechart là gì?"</t>
+  </si>
+  <si>
+    <t>"Các kịch bản (scenarios) được mô tả trên Sequence Diagram đóng vai trò gì trong giai đoạn Kiểm thử tích hợp (Integration Testing) theo phương pháp COMET?"</t>
+  </si>
+  <si>
+    <t>"Tại sao phương pháp COMET lại đánh giá Communication Diagram cao hơn Sequence Diagram khi chuyển từ giai đoạn Phân tích (Analysis) sang Thiết kế kiến trúc (Architectural Design)? Nếu chỉ có Sequence Diagram, ta phải làm thêm bước trung gian nào?"</t>
+  </si>
+  <si>
+    <t>"Việc đánh số thứ tự thông điệp (ví dụ: 1.1, 1.2) trên Sequence Diagram có thực sự bắt buộc không? Tại sao trong các dự án thực tế, người ta vẫn thường xuyên ghi số thứ tự này?"</t>
+  </si>
+  <si>
+    <t>"Làm thế nào để biểu diễn cả kịch bản chính (main sequence) và kịch bản lỗi/thay thế (alternative sequences) trên cùng một 'Generic Sequence Diagram'? Hạn chế của cách làm này là gì?"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Giải thích rõ trong phương pháp COMET, khi chuyển từ Analysis sang Design model, các thông điệp (messages) trên Sequence Diagram thay đổi từ mức ý niệm/logic sang đặc tả kỹ thuật: (1) Biến các message thành lời gọi hàm thực tế có đầy đủ tham số và giá trị trả về; (2) Định rõ cơ chế đồng bộ (Synchronous) hoặc bất đồng bộ (Asynchronous) dựa trên việc phân loại đối tượng là Active Object (Thread) hay Passive Object; (3) Xuất hiện thêm các thông điệp điều khiển hạ tầng (start/stop thread, exception).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Áp dụng tư duy này vào dự án thực tế để chuẩn hóa sơ đồ thiết kế; khi vẽ Design Sequence Diagram bắt buộc phải phân loại rõ Active/Passive Object, chuyển toàn bộ message thành tên hàm cụ thể và dùng đúng loại mũi tên biểu diễn cơ chế đồng bộ nhằm đảm bảo tính khả thi khi code.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Định nghĩa Generic Sequence Diagram là sơ đồ biểu diễn tất cả các kịch bản có thể xảy ra của một Use Case. Để gom cả kịch bản chính và kịch bản thay thế vào cùng một sơ đồ, UML sử dụng các khối tương tác (Combined Fragments). Trong đó: Khối alt (Alternatives) đóng vai trò như câu lệnh điều kiện if/else, chia sơ đồ thành các nhánh độc lập, chỉ một nhánh được thực thi tùy thuộc vào điều kiện (guard condition); khối loop (Loop) đóng vai trò như vòng lặp for/while, dùng để lặp lại một chuỗi thông điệp cho đến khi điều kiện dừng thỏa mãn.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Thấu hiểu cách dùng các khối điều khiển alt và loop để tối ưu hóa việc thiết kế sơ đồ; áp dụng ngay vào dự án bằng cách tích hợp các kịch bản ngoại lệ (sai mật khẩu, hết hàng, lỗi hệ thống) và luồng lặp dữ liệu vào chung một sơ đồ Generic Sequence Diagram thay vì vẽ rời rạc, giúp tài liệu thiết kế gọn gàng, bao quát và logic hơn.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Định nghĩa State-Dependent Dynamic Interaction Modeling là sự kết hợp giữa luồng trao đổi thông điệp và trạng thái nội tại của đối tượng điều khiển (Control Object). Mối quan hệ cốt lõi giữa hai sơ đồ được thể hiện qua cơ chế kích hoạt và phản hồi: Một thông điệp (message) gửi đến Control Object trên Sequence Diagram sẽ đóng vai trò là một sự kiện (event) kích hoạt sự chuyển dịch trạng thái (transition) trên Statechart Diagram; ngược lại, hành động (action) được thực thi trên Statechart sau khi chuyển trạng thái sẽ chính là các thông điệp (messages) tiếp theo mà Control Object gửi đi cho các đối tượng khác trên Sequence Diagram.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nắm vững mối liên kết chặt chẽ giữa hai loại sơ đồ để đảm bảo tính nhất quán (consistency) khi thiết kế hệ thống phụ thuộc trạng thái; áp dụng vào dự án bằng cách luôn kiểm tra chéo (cross-check): mỗi khi vẽ một message gửi tới Control Object trên Sequence Diagram, phải đảm bảo Statechart của nó có một Event tương ứng, và các Action trên Statechart phải khớp với các message đầu ra trên Sequence Diagram.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Định nghĩa vai trò cốt lõi của Sequence Diagram trong COMET là làm căn cứ (baseline) định hình các kịch bản kiểm thử tích hợp. Vì Sequence Diagram thể hiện rõ luồng tương tác giữa các thành phần (Boundary, Control, Entity), nên trong Integration Testing, mỗi kịch bản (scenario) trên sơ đồ sẽ trực tiếp biến thành một Integration Test Case. Luồng đi của các thông điệp (messages) chính là trình tự các bước thực thi (test steps) và dữ liệu truyền vào; trong khi kết quả đầu ra hoặc sự thay đổi trạng thái của đối tượng đích chính là kết quả mong đợi (expected results) để nghiệm thu việc tích hợp giữa các module/thread.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Thấu hiểu giá trị của sơ đồ tương tác không chỉ dừng ở bước thiết kế mà còn phục vụ trực tiếp cho QA/Tester; áp dụng vào dự án bằng cách chuyển giao các sơ đồ Sequence Diagram cho đội kiểm thử ngay khi hoàn thiện thiết kế, sử dụng các nhánh alt (kịch bản thay thế/ngoại lệ) để xây dựng bộ test case bao phủ toàn bộ các lỗi tích hợp có thể xảy ra giữa các subsystem.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Giải thích lý do COMET ưu tiên Communication Diagram ở bước thiết kế kiến trúc vì sơ đồ này có cấu trúc dạng mạng lưới (network-oriented), làm nổi bật mối quan hệ cấu trúc vững chắc và các kênh giao tiếp giữa các đối tượng; từ đó giúp kiến trúc sư dễ dàng gom nhóm các đối tượng liên quan thành các Subsystem (Phân hệ) hoặc Task/Thread (Tiến trình đồng thời). Nếu chỉ có Sequence Diagram (vốn tập trung vào trình tự thời gian của một kịch bản đơn lẻ), ta bắt buộc phải làm thêm một bước trung gian là "Tổng hợp luồng" (Consolidation): gom tất cả các Sequence Diagram rời rạc của các Use Case lại để tạo ra một góc nhìn tổng thể về cấu trúc và các liên kết tĩnh giữa các đối tượng trước khi phân rã kiến trúc.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nắm vững thế mạnh của từng loại sơ đồ để chọn lựa công cụ trực quan hóa phù hợp cho từng giai đoạn; áp dụng vào dự án bằng cách sử dụng Sequence Diagram khi cần làm việc với khách hàng/PO để làm rõ luồng nghiệp vụ, nhưng khi họp kỹ thuật để phân chia module/kiến trúc backend (Microservices, Task Allocation) thì sẽ chuyển đổi sang Communication Diagram để có cái nhìn bao quát về hạ tầng kết nối.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Làm rõ quy chuẩn UML: Việc đánh số thứ tự thông điệp (như 1.1, 1.2) trên Sequence Diagram không bắt buộc (vì trục thời gian từ trên xuống dưới đã thể hiện trình tự). Tuy nhiên, các dự án thực tế vẫn thường xuyên ghi số thứ tự vì 3 lý do cốt lõi: (1) Giúp theo dõi chính xác các luồng lồng nhau (nested calls) hoặc các nhánh điều kiện alt/else phức tạp; (2) Giúp giao tiếp, thảo luận nhóm (Code Review, Design Review) dễ dàng bằng cách chỉ đích danh mã số thông điệp; (3) Hỗ trợ ánh xạ (traceability) trực tiếp sang mã nguồn hoặc các bước kiểm thử (test steps) trong Integration Test.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nhận thức rõ sự khác biệt giữa lý thuyết chuẩn hóa và thực tế vận hành dự án để linh hoạt áp dụng; quyết định sẽ chủ động đánh số thứ tự thông điệp cho các sơ đồ Sequence Diagram có luồng xử lý phức tạp, nhiều nhánh rẽ hoặc xử lý bất đồng bộ trong dự án, giúp đội ngũ lập trình viên và kiểm thử dễ dàng đọc hiểu, hạn chế tối đa việc hiểu lầm tài liệu thiết kế.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Giải thích phương pháp biểu diễn tích hợp trên Generic Sequence Diagram bằng cách sử dụng các khối tương tác alt (Alternatives) để chia sơ đồ thành các phân đoạn điều kiện (mỗi phân đoạn đại diện cho kịch bản chính hoặc một kịch bản lỗi kèm điều kiện ràng buộc [guard]). Tuy nhiên, cách làm này có hạn chế lớn là: Khi hệ thống có quá nhiều kịch bản thay thế/ngoại lệ, sơ đồ sẽ trở nên cực kỳ phức tạp, xuất hiện các khối alt lồng nhau (nested), gây ra tình trạng "quá tải thông tin" (visual clutter), làm giảm tính trực quan và rất khó bảo trì hoặc cập nhật khi logic nghiệp vụ thay đổi.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Thấu hiểu ranh giới giữa việc tối ưu hóa sơ đồ và việc gây quá tải thông tin để áp dụng linh hoạt; quyết định trong dự án thực tế sẽ chỉ gom kịch bản chính và các kịch bản lỗi phổ biến, quan trọng (ví dụ: lỗi validate, lỗi xác thực) vào chung một Generic Sequence Diagram. Đối với các luồng ngoại lệ quá phức tạp hoặc mang tính kỹ thuật sâu, sẽ tách ra thành các sơ đồ Sequence Diagram riêng biệt để giữ cho tài liệu thiết kế luôn sáng sủa, dễ đọc.</t>
     </r>
   </si>
 </sst>
@@ -1026,13 +1369,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1123,7 +1473,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1137,7 +1487,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1152,50 +1502,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1982,4 +2338,132 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0658147-FBE4-494E-A01E-50377A78CF9D}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="31.88671875" customWidth="1"/>
+    <col min="3" max="3" width="36.88671875" customWidth="1"/>
+    <col min="4" max="4" width="56.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="243" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="253.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="268.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="302.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="256.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="244.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="246" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>